<commit_message>
Daily EOD data and reports for 2026-08-14
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260814.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260814.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.535</v>
+        <v>1.537</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.04</v>
+        <v>-0.038</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-2.54%</t>
+          <t>-2.41%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>235132.83</v>
+        <v>235439.2</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-6127.24</v>
+        <v>-5820.88</v>
       </c>
     </row>
     <row r="5">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>61.07</v>
+        <v>61.02</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-2.38</v>
+        <v>-2.43</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-3.75%</t>
+          <t>-3.83%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>675739.55</v>
+        <v>675186.3</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-26334.7</v>
+        <v>-26887.95</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>169.3</v>
+        <v>169</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.18%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>136.89</v>
+        <v>137.02</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0.63</v>
+        <v>-0.5</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.46%</t>
+          <t>-0.36%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>547560</v>
+        <v>548080</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-2520</v>
+        <v>-2000</v>
       </c>
     </row>
     <row r="12">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>35.5</v>
+        <v>35.46</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.24</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.56%</t>
+          <t>-0.67%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1749186.83</v>
+        <v>1749459.95</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-35543.2</v>
+        <v>-35270.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>